<commit_message>
CM and CWM figures updated with significances from LMs
</commit_message>
<xml_diff>
--- a/results/CM vs microclimatic gradients.xlsx
+++ b/results/CM vs microclimatic gradients.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="17745" windowHeight="14670"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="17745" windowHeight="14670" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="CM vs micro MED" sheetId="1" r:id="rId1"/>
@@ -981,22 +981,22 @@
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="8" t="s">
-        <v>6</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="C3" s="2">
-        <v>1.8233142963540399E-5</v>
-      </c>
-      <c r="D3" s="2">
-        <v>1.08031995996393E-5</v>
+        <v>16</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C3" s="1">
+        <v>-3.6072578934203299E-3</v>
+      </c>
+      <c r="D3" s="1">
+        <v>1.2690195160271101E-3</v>
       </c>
       <c r="E3" s="1">
-        <v>1.6877539654223499</v>
-      </c>
-      <c r="F3" s="1">
-        <v>9.8228581389421102E-2</v>
+        <v>-2.8425550969566702</v>
+      </c>
+      <c r="F3" s="4">
+        <v>6.6521005502137602E-3</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
@@ -1004,147 +1004,147 @@
       <c r="B4" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="C4" s="2">
-        <v>2.0349472277592401E-5</v>
+      <c r="C4" s="1">
+        <v>-1.4862568015520301E-4</v>
       </c>
       <c r="D4" s="1">
-        <v>1.3714869420665001E-4</v>
+        <v>1.4049986044080099E-3</v>
       </c>
       <c r="E4" s="1">
-        <v>0.148375253554588</v>
+        <v>-0.105783507320868</v>
       </c>
       <c r="F4" s="1">
-        <v>0.88269515722479497</v>
+        <v>0.91621408320581599</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="8"/>
-      <c r="B5" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="C5" s="1">
-        <v>-2.4835389120634401E-4</v>
+      <c r="B5" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C5" s="2">
+        <v>5.2599606029830298E-5</v>
       </c>
       <c r="D5" s="1">
-        <v>1.23875119163699E-4</v>
+        <v>1.10671708895486E-4</v>
       </c>
       <c r="E5" s="1">
-        <v>-2.0048730760706501</v>
-      </c>
-      <c r="F5" s="3">
-        <v>5.0882349685987899E-2</v>
+        <v>0.475275990176528</v>
+      </c>
+      <c r="F5" s="1">
+        <v>0.63683937849943295</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" s="8"/>
-      <c r="B6" s="1" t="s">
+      <c r="B6" s="3" t="s">
         <v>10</v>
       </c>
       <c r="C6" s="1">
-        <v>1.1983767405981699E-4</v>
-      </c>
-      <c r="D6" s="2">
-        <v>7.8823798345412999E-5</v>
+        <v>1.50116471133251E-3</v>
+      </c>
+      <c r="D6" s="1">
+        <v>8.0749822162049705E-4</v>
       </c>
       <c r="E6" s="1">
-        <v>1.520323513651</v>
-      </c>
-      <c r="F6" s="1">
-        <v>0.13527418652671999</v>
+        <v>1.85903160049066</v>
+      </c>
+      <c r="F6" s="3">
+        <v>6.9426541584144894E-2</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A7" s="8" t="s">
-        <v>11</v>
-      </c>
-      <c r="B7" s="1" t="s">
+      <c r="A7" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C7" s="1">
+        <v>-9.7186664867520405E-3</v>
+      </c>
+      <c r="D7" s="1">
+        <v>3.37966265215105E-3</v>
+      </c>
+      <c r="E7" s="1">
+        <v>-2.8756321227997201</v>
+      </c>
+      <c r="F7" s="4">
+        <v>6.0899396888603203E-3</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A8" s="10"/>
+      <c r="B8" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C8" s="1">
+        <v>-2.96547411479808E-3</v>
+      </c>
+      <c r="D8" s="1">
+        <v>3.7418032186832401E-3</v>
+      </c>
+      <c r="E8" s="1">
+        <v>-0.792525405930256</v>
+      </c>
+      <c r="F8" s="1">
+        <v>0.43212287909522301</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A9" s="10"/>
+      <c r="B9" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="C7" s="1">
-        <v>-1.1152605499439199E-3</v>
-      </c>
-      <c r="D7" s="1">
-        <v>6.4520745454109505E-4</v>
-      </c>
-      <c r="E7" s="1">
-        <v>-1.72853016823427</v>
-      </c>
-      <c r="F7" s="1">
-        <v>9.0600955728569299E-2</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A8" s="8"/>
-      <c r="B8" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="C8" s="1">
-        <v>-2.0343295228709299E-2</v>
-      </c>
-      <c r="D8" s="1">
-        <v>8.1910325794278798E-3</v>
-      </c>
-      <c r="E8" s="1">
-        <v>-2.4836057031200598</v>
-      </c>
-      <c r="F8" s="4">
-        <v>1.6711393192260102E-2</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A9" s="8"/>
-      <c r="B9" s="1" t="s">
-        <v>9</v>
-      </c>
       <c r="C9" s="1">
-        <v>1.5479634490939999E-3</v>
+        <v>6.1703022608801503E-4</v>
       </c>
       <c r="D9" s="1">
-        <v>7.3982850709574796E-3</v>
+        <v>2.9474175651355102E-4</v>
       </c>
       <c r="E9" s="1">
-        <v>0.209232738972258</v>
-      </c>
-      <c r="F9" s="1">
-        <v>0.83519040955672696</v>
+        <v>2.0934605038212402</v>
+      </c>
+      <c r="F9" s="4">
+        <v>4.1849565675452997E-2</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A10" s="8"/>
+      <c r="A10" s="10"/>
       <c r="B10" s="1" t="s">
         <v>10</v>
       </c>
       <c r="C10" s="1">
-        <v>-6.6518676371898899E-3</v>
+        <v>2.6048141438072699E-3</v>
       </c>
       <c r="D10" s="1">
-        <v>4.7076518228361302E-3</v>
+        <v>2.1505355487621098E-3</v>
       </c>
       <c r="E10" s="1">
-        <v>-1.4129905709939401</v>
+        <v>1.2112397515617199</v>
       </c>
       <c r="F10" s="1">
-        <v>0.164389493719657</v>
+        <v>0.23198952469817799</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="B11" s="1" t="s">
-        <v>7</v>
+      <c r="B11" s="4" t="s">
+        <v>9</v>
       </c>
       <c r="C11" s="1">
-        <v>2.3166489008347299E-4</v>
+        <v>-9.6861009576420208E-3</v>
       </c>
       <c r="D11" s="1">
-        <v>1.91826578163541E-4</v>
+        <v>2.19958355944536E-3</v>
       </c>
       <c r="E11" s="1">
-        <v>1.20767879144447</v>
-      </c>
-      <c r="F11" s="1">
-        <v>0.233343635342591</v>
+        <v>-4.4036067263952603</v>
+      </c>
+      <c r="F11" s="5">
+        <v>6.2977067874974701E-5</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
@@ -1167,20 +1167,20 @@
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" s="8"/>
-      <c r="B13" s="4" t="s">
-        <v>9</v>
+      <c r="B13" s="1" t="s">
+        <v>7</v>
       </c>
       <c r="C13" s="1">
-        <v>-9.6861009576420208E-3</v>
+        <v>2.3166489008347299E-4</v>
       </c>
       <c r="D13" s="1">
-        <v>2.19958355944536E-3</v>
+        <v>1.91826578163541E-4</v>
       </c>
       <c r="E13" s="1">
-        <v>-4.4036067263952603</v>
-      </c>
-      <c r="F13" s="5">
-        <v>6.2977067874974701E-5</v>
+        <v>1.20767879144447</v>
+      </c>
+      <c r="F13" s="1">
+        <v>0.233343635342591</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
@@ -1203,22 +1203,22 @@
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" s="8" t="s">
-        <v>13</v>
-      </c>
-      <c r="B15" s="1" t="s">
-        <v>7</v>
+        <v>6</v>
+      </c>
+      <c r="B15" s="3" t="s">
+        <v>9</v>
       </c>
       <c r="C15" s="1">
-        <v>-1.7997596633955601E-4</v>
+        <v>-2.4835389120634401E-4</v>
       </c>
       <c r="D15" s="1">
-        <v>2.1761152063240002E-3</v>
+        <v>1.23875119163699E-4</v>
       </c>
       <c r="E15" s="1">
-        <v>-8.2705164605499204E-2</v>
-      </c>
-      <c r="F15" s="1">
-        <v>0.93444482661378703</v>
+        <v>-2.0048730760706501</v>
+      </c>
+      <c r="F15" s="3">
+        <v>5.0882349685987899E-2</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
@@ -1226,35 +1226,35 @@
       <c r="B16" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="C16" s="1">
-        <v>2.9038975186392601E-2</v>
+      <c r="C16" s="2">
+        <v>2.0349472277592401E-5</v>
       </c>
       <c r="D16" s="1">
-        <v>2.76262005749238E-2</v>
+        <v>1.3714869420665001E-4</v>
       </c>
       <c r="E16" s="1">
-        <v>1.0511389399218101</v>
+        <v>0.148375253554588</v>
       </c>
       <c r="F16" s="1">
-        <v>0.29868563930830799</v>
+        <v>0.88269515722479497</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17" s="8"/>
       <c r="B17" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="C17" s="1">
-        <v>2.9569378756749299E-2</v>
-      </c>
-      <c r="D17" s="1">
-        <v>2.4952471535037001E-2</v>
+        <v>7</v>
+      </c>
+      <c r="C17" s="2">
+        <v>1.8233142963540399E-5</v>
+      </c>
+      <c r="D17" s="2">
+        <v>1.08031995996393E-5</v>
       </c>
       <c r="E17" s="1">
-        <v>1.18502805284156</v>
+        <v>1.6877539654223499</v>
       </c>
       <c r="F17" s="1">
-        <v>0.24209258446117399</v>
+        <v>9.8228581389421102E-2</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.25">
@@ -1263,72 +1263,72 @@
         <v>10</v>
       </c>
       <c r="C18" s="1">
-        <v>-6.3905265837868796E-3</v>
-      </c>
-      <c r="D18" s="1">
-        <v>1.5877672592978499E-2</v>
+        <v>1.1983767405981699E-4</v>
+      </c>
+      <c r="D18" s="2">
+        <v>7.8823798345412999E-5</v>
       </c>
       <c r="E18" s="1">
-        <v>-0.40248509637444702</v>
+        <v>1.520323513651</v>
       </c>
       <c r="F18" s="1">
-        <v>0.68919137950349796</v>
+        <v>0.13527418652671999</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A19" s="8" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="C19" s="1">
-        <v>6.1875044666251204E-4</v>
+        <v>1.5479634490939999E-3</v>
       </c>
       <c r="D19" s="1">
-        <v>2.0282397086816301E-3</v>
+        <v>7.3982850709574796E-3</v>
       </c>
       <c r="E19" s="1">
-        <v>0.30506771167827301</v>
+        <v>0.209232738972258</v>
       </c>
       <c r="F19" s="1">
-        <v>0.76169070210021295</v>
+        <v>0.83519040955672696</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20" s="8"/>
-      <c r="B20" s="1" t="s">
+      <c r="B20" s="4" t="s">
         <v>8</v>
       </c>
       <c r="C20" s="1">
-        <v>-5.7096452452447301E-3</v>
+        <v>-2.0343295228709299E-2</v>
       </c>
       <c r="D20" s="1">
-        <v>2.5748892725544901E-2</v>
+        <v>8.1910325794278798E-3</v>
       </c>
       <c r="E20" s="1">
-        <v>-0.22174333110566499</v>
-      </c>
-      <c r="F20" s="1">
-        <v>0.82549518635725805</v>
+        <v>-2.4836057031200598</v>
+      </c>
+      <c r="F20" s="4">
+        <v>1.6711393192260102E-2</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A21" s="8"/>
-      <c r="B21" s="3" t="s">
-        <v>9</v>
+      <c r="B21" s="1" t="s">
+        <v>7</v>
       </c>
       <c r="C21" s="1">
-        <v>4.4088729294911803E-2</v>
+        <v>-1.1152605499439199E-3</v>
       </c>
       <c r="D21" s="1">
-        <v>2.3256853979988699E-2</v>
+        <v>6.4520745454109505E-4</v>
       </c>
       <c r="E21" s="1">
-        <v>1.89573058044944</v>
-      </c>
-      <c r="F21" s="3">
-        <v>6.4288284198534898E-2</v>
+        <v>-1.72853016823427</v>
+      </c>
+      <c r="F21" s="1">
+        <v>9.0600955728569299E-2</v>
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.25">
@@ -1337,36 +1337,36 @@
         <v>10</v>
       </c>
       <c r="C22" s="1">
-        <v>-2.7282682462299803E-4</v>
+        <v>-6.6518676371898899E-3</v>
       </c>
       <c r="D22" s="1">
-        <v>1.47987229448781E-2</v>
+        <v>4.7076518228361302E-3</v>
       </c>
       <c r="E22" s="1">
-        <v>-1.8435835689283201E-2</v>
+        <v>-1.4129905709939401</v>
       </c>
       <c r="F22" s="1">
-        <v>0.98537089879256601</v>
+        <v>0.164389493719657</v>
       </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A23" s="8" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="C23" s="1">
-        <v>-7.2151906794048603E-4</v>
+        <v>2.9569378756749299E-2</v>
       </c>
       <c r="D23" s="1">
-        <v>1.2874441249869999E-3</v>
+        <v>2.4952471535037001E-2</v>
       </c>
       <c r="E23" s="1">
-        <v>-0.56042748103555196</v>
+        <v>1.18502805284156</v>
       </c>
       <c r="F23" s="1">
-        <v>0.57790738199043301</v>
+        <v>0.24209258446117399</v>
       </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.25">
@@ -1375,34 +1375,34 @@
         <v>8</v>
       </c>
       <c r="C24" s="1">
-        <v>-1.4775078079508E-2</v>
+        <v>2.9038975186392601E-2</v>
       </c>
       <c r="D24" s="1">
-        <v>1.6344350484081199E-2</v>
+        <v>2.76262005749238E-2</v>
       </c>
       <c r="E24" s="1">
-        <v>-0.90398686040772402</v>
+        <v>1.0511389399218101</v>
       </c>
       <c r="F24" s="1">
-        <v>0.37071241321783299</v>
+        <v>0.29868563930830799</v>
       </c>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A25" s="8"/>
-      <c r="B25" s="4" t="s">
-        <v>9</v>
+      <c r="B25" s="1" t="s">
+        <v>7</v>
       </c>
       <c r="C25" s="1">
-        <v>5.8825892885889103E-2</v>
+        <v>-1.7997596633955601E-4</v>
       </c>
       <c r="D25" s="1">
-        <v>1.47625055825771E-2</v>
+        <v>2.1761152063240002E-3</v>
       </c>
       <c r="E25" s="1">
-        <v>3.9848176555690098</v>
-      </c>
-      <c r="F25" s="4">
-        <v>2.3896406994294701E-4</v>
+        <v>-8.2705164605499204E-2</v>
+      </c>
+      <c r="F25" s="1">
+        <v>0.93444482661378703</v>
       </c>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.25">
@@ -1411,36 +1411,36 @@
         <v>10</v>
       </c>
       <c r="C26" s="1">
-        <v>-1.37319352158409E-2</v>
+        <v>-6.3905265837868796E-3</v>
       </c>
       <c r="D26" s="1">
-        <v>9.3936278000778892E-3</v>
+        <v>1.5877672592978499E-2</v>
       </c>
       <c r="E26" s="1">
-        <v>-1.4618351405968</v>
+        <v>-0.40248509637444702</v>
       </c>
       <c r="F26" s="1">
-        <v>0.150584814092001</v>
+        <v>0.68919137950349796</v>
       </c>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A27" s="8" t="s">
-        <v>16</v>
-      </c>
-      <c r="B27" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="C27" s="2">
-        <v>5.2599606029830298E-5</v>
+        <v>14</v>
+      </c>
+      <c r="B27" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="C27" s="1">
+        <v>4.4088729294911803E-2</v>
       </c>
       <c r="D27" s="1">
-        <v>1.10671708895486E-4</v>
+        <v>2.3256853979988699E-2</v>
       </c>
       <c r="E27" s="1">
-        <v>0.475275990176528</v>
-      </c>
-      <c r="F27" s="1">
-        <v>0.63683937849943295</v>
+        <v>1.89573058044944</v>
+      </c>
+      <c r="F27" s="3">
+        <v>6.4288284198534898E-2</v>
       </c>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.25">
@@ -1449,138 +1449,138 @@
         <v>8</v>
       </c>
       <c r="C28" s="1">
-        <v>-1.4862568015520301E-4</v>
+        <v>-5.7096452452447301E-3</v>
       </c>
       <c r="D28" s="1">
-        <v>1.4049986044080099E-3</v>
+        <v>2.5748892725544901E-2</v>
       </c>
       <c r="E28" s="1">
-        <v>-0.105783507320868</v>
+        <v>-0.22174333110566499</v>
       </c>
       <c r="F28" s="1">
-        <v>0.91621408320581599</v>
+        <v>0.82549518635725805</v>
       </c>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A29" s="8"/>
-      <c r="B29" s="4" t="s">
-        <v>9</v>
+      <c r="B29" s="1" t="s">
+        <v>7</v>
       </c>
       <c r="C29" s="1">
-        <v>-3.6072578934203299E-3</v>
+        <v>6.1875044666251204E-4</v>
       </c>
       <c r="D29" s="1">
-        <v>1.2690195160271101E-3</v>
+        <v>2.0282397086816301E-3</v>
       </c>
       <c r="E29" s="1">
-        <v>-2.8425550969566702</v>
-      </c>
-      <c r="F29" s="4">
-        <v>6.6521005502137602E-3</v>
+        <v>0.30506771167827301</v>
+      </c>
+      <c r="F29" s="1">
+        <v>0.76169070210021295</v>
       </c>
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A30" s="8"/>
-      <c r="B30" s="3" t="s">
+      <c r="B30" s="1" t="s">
         <v>10</v>
       </c>
       <c r="C30" s="1">
-        <v>1.50116471133251E-3</v>
+        <v>-2.7282682462299803E-4</v>
       </c>
       <c r="D30" s="1">
-        <v>8.0749822162049705E-4</v>
+        <v>1.47987229448781E-2</v>
       </c>
       <c r="E30" s="1">
-        <v>1.85903160049066</v>
-      </c>
-      <c r="F30" s="3">
-        <v>6.9426541584144894E-2</v>
+        <v>-1.8435835689283201E-2</v>
+      </c>
+      <c r="F30" s="1">
+        <v>0.98537089879256601</v>
       </c>
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A31" s="10" t="s">
-        <v>17</v>
+      <c r="A31" s="8" t="s">
+        <v>15</v>
       </c>
       <c r="B31" s="4" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="C31" s="1">
-        <v>6.1703022608801503E-4</v>
+        <v>5.8825892885889103E-2</v>
       </c>
       <c r="D31" s="1">
-        <v>2.9474175651355102E-4</v>
+        <v>1.47625055825771E-2</v>
       </c>
       <c r="E31" s="1">
-        <v>2.0934605038212402</v>
+        <v>3.9848176555690098</v>
       </c>
       <c r="F31" s="4">
-        <v>4.1849565675452997E-2</v>
+        <v>2.3896406994294701E-4</v>
       </c>
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A32" s="10"/>
+      <c r="A32" s="8"/>
       <c r="B32" s="1" t="s">
         <v>8</v>
       </c>
       <c r="C32" s="1">
-        <v>-2.96547411479808E-3</v>
+        <v>-1.4775078079508E-2</v>
       </c>
       <c r="D32" s="1">
-        <v>3.7418032186832401E-3</v>
+        <v>1.6344350484081199E-2</v>
       </c>
       <c r="E32" s="1">
-        <v>-0.792525405930256</v>
+        <v>-0.90398686040772402</v>
       </c>
       <c r="F32" s="1">
-        <v>0.43212287909522301</v>
+        <v>0.37071241321783299</v>
       </c>
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A33" s="10"/>
-      <c r="B33" s="4" t="s">
-        <v>9</v>
+      <c r="A33" s="8"/>
+      <c r="B33" s="1" t="s">
+        <v>7</v>
       </c>
       <c r="C33" s="1">
-        <v>-9.7186664867520405E-3</v>
+        <v>-7.2151906794048603E-4</v>
       </c>
       <c r="D33" s="1">
-        <v>3.37966265215105E-3</v>
+        <v>1.2874441249869999E-3</v>
       </c>
       <c r="E33" s="1">
-        <v>-2.8756321227997201</v>
-      </c>
-      <c r="F33" s="4">
-        <v>6.0899396888603203E-3</v>
+        <v>-0.56042748103555196</v>
+      </c>
+      <c r="F33" s="1">
+        <v>0.57790738199043301</v>
       </c>
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A34" s="10"/>
+      <c r="A34" s="8"/>
       <c r="B34" s="1" t="s">
         <v>10</v>
       </c>
       <c r="C34" s="1">
-        <v>2.6048141438072699E-3</v>
+        <v>-1.37319352158409E-2</v>
       </c>
       <c r="D34" s="1">
-        <v>2.1505355487621098E-3</v>
+        <v>9.3936278000778892E-3</v>
       </c>
       <c r="E34" s="1">
-        <v>1.2112397515617199</v>
+        <v>-1.4618351405968</v>
       </c>
       <c r="F34" s="1">
-        <v>0.23198952469817799</v>
+        <v>0.150584814092001</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="9">
+    <mergeCell ref="A19:A22"/>
+    <mergeCell ref="A15:A18"/>
+    <mergeCell ref="A1:F1"/>
     <mergeCell ref="A7:A10"/>
     <mergeCell ref="A3:A6"/>
-    <mergeCell ref="A1:F1"/>
     <mergeCell ref="A31:A34"/>
     <mergeCell ref="A27:A30"/>
     <mergeCell ref="A23:A26"/>
-    <mergeCell ref="A19:A22"/>
-    <mergeCell ref="A15:A18"/>
     <mergeCell ref="A11:A14"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1628,22 +1628,22 @@
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="8" t="s">
-        <v>6</v>
-      </c>
-      <c r="B3" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="C3" s="2">
-        <v>1.3575622868601501E-5</v>
-      </c>
-      <c r="D3" s="2">
-        <v>6.1456258488287402E-6</v>
+        <v>16</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C3" s="1">
+        <v>-3.64146958916518E-4</v>
+      </c>
+      <c r="D3" s="1">
+        <v>2.7071371014617701E-4</v>
       </c>
       <c r="E3" s="1">
-        <v>2.2089894833394101</v>
-      </c>
-      <c r="F3" s="4">
-        <v>3.2684032924149502E-2</v>
+        <v>-1.34513674508724</v>
+      </c>
+      <c r="F3" s="1">
+        <v>0.185799557133072</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
@@ -1651,35 +1651,35 @@
       <c r="B4" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="C4" s="2">
-        <v>-5.8390208894141502E-5</v>
-      </c>
-      <c r="D4" s="2">
-        <v>4.0125816043901601E-5</v>
+      <c r="C4" s="1">
+        <v>-2.7141891938760603E-4</v>
+      </c>
+      <c r="D4" s="1">
+        <v>5.7390735534695305E-4</v>
       </c>
       <c r="E4" s="1">
-        <v>-1.4551781035495199</v>
+        <v>-0.47293159228377701</v>
       </c>
       <c r="F4" s="1">
-        <v>0.15305398014178601</v>
+        <v>0.63871063739713796</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="8"/>
-      <c r="B5" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="C5" s="2">
-        <v>-3.5825154663033903E-5</v>
+      <c r="B5" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C5" s="1">
+        <v>3.6091968136373401E-4</v>
       </c>
       <c r="D5" s="2">
-        <v>1.8927460038076501E-5</v>
+        <v>8.7899019274630306E-5</v>
       </c>
       <c r="E5" s="1">
-        <v>-1.89276081370476</v>
-      </c>
-      <c r="F5" s="3">
-        <v>6.5294653231981498E-2</v>
+        <v>4.1060717666949396</v>
+      </c>
+      <c r="F5" s="4">
+        <v>1.8169073902427901E-4</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
@@ -1688,72 +1688,72 @@
         <v>10</v>
       </c>
       <c r="C6" s="2">
-        <v>-3.0176903192067899E-5</v>
-      </c>
-      <c r="D6" s="2">
-        <v>2.84183722426402E-5</v>
+        <v>-6.1139804463442406E-5</v>
+      </c>
+      <c r="D6" s="1">
+        <v>4.0645934376000399E-4</v>
       </c>
       <c r="E6" s="1">
-        <v>-1.06188007301801</v>
+        <v>-0.150420467390074</v>
       </c>
       <c r="F6" s="1">
-        <v>0.29435811396760603</v>
+        <v>0.88115298754952798</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" s="8" t="s">
-        <v>11</v>
-      </c>
-      <c r="B7" s="3" t="s">
-        <v>7</v>
+        <v>17</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>9</v>
       </c>
       <c r="C7" s="1">
-        <v>-5.5751340316831095E-4</v>
+        <v>1.4546674291028201E-3</v>
       </c>
       <c r="D7" s="1">
-        <v>3.1191178968292902E-4</v>
+        <v>5.1215711657116403E-4</v>
       </c>
       <c r="E7" s="1">
-        <v>-1.7874072786252999</v>
-      </c>
-      <c r="F7" s="3">
-        <v>8.1089298193969594E-2</v>
+        <v>2.8402757318724001</v>
+      </c>
+      <c r="F7" s="4">
+        <v>6.9216450943544302E-3</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" s="8"/>
-      <c r="B8" s="4" t="s">
+      <c r="B8" s="1" t="s">
         <v>8</v>
       </c>
       <c r="C8" s="1">
-        <v>-7.5561135023714298E-3</v>
+        <v>5.7953254205743605E-4</v>
       </c>
       <c r="D8" s="1">
-        <v>2.03652409089086E-3</v>
+        <v>1.08576228420335E-3</v>
       </c>
       <c r="E8" s="1">
-        <v>-3.7102991003981001</v>
-      </c>
-      <c r="F8" s="4">
-        <v>6.0210191906117001E-4</v>
+        <v>0.53375637604013104</v>
+      </c>
+      <c r="F8" s="1">
+        <v>0.59632390024812099</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" s="8"/>
-      <c r="B9" s="4" t="s">
-        <v>9</v>
+      <c r="B9" s="1" t="s">
+        <v>7</v>
       </c>
       <c r="C9" s="1">
-        <v>2.15160279809898E-3</v>
+        <v>1.6039099443968701E-4</v>
       </c>
       <c r="D9" s="1">
-        <v>9.6063412902913897E-4</v>
+        <v>1.66294157162633E-4</v>
       </c>
       <c r="E9" s="1">
-        <v>2.2397734299462102</v>
-      </c>
-      <c r="F9" s="4">
-        <v>3.0456337762944499E-2</v>
+        <v>0.96450168289934102</v>
+      </c>
+      <c r="F9" s="1">
+        <v>0.34031531873463899</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
@@ -1761,37 +1761,37 @@
       <c r="B10" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="C10" s="2">
-        <v>3.5716593827619803E-5</v>
+      <c r="C10" s="1">
+        <v>-7.5215013217949395E-4</v>
       </c>
       <c r="D10" s="1">
-        <v>1.4423307835713601E-3</v>
+        <v>7.6897119614342802E-4</v>
       </c>
       <c r="E10" s="1">
-        <v>2.47631085978639E-2</v>
+        <v>-0.97812523531662099</v>
       </c>
       <c r="F10" s="1">
-        <v>0.98036120027870799</v>
+        <v>0.33361305843751698</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="B11" s="3" t="s">
-        <v>7</v>
+      <c r="B11" s="1" t="s">
+        <v>9</v>
       </c>
       <c r="C11" s="1">
-        <v>3.2791453922484702E-4</v>
+        <v>1.97028826221731E-4</v>
       </c>
       <c r="D11" s="1">
-        <v>1.91218155012373E-4</v>
+        <v>5.8891870032100595E-4</v>
       </c>
       <c r="E11" s="1">
-        <v>1.7148713687967001</v>
-      </c>
-      <c r="F11" s="3">
-        <v>9.3739580007072595E-2</v>
+        <v>0.33456031556534899</v>
+      </c>
+      <c r="F11" s="1">
+        <v>0.73962183969531003</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
@@ -1814,20 +1814,20 @@
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" s="8"/>
-      <c r="B13" s="1" t="s">
-        <v>9</v>
+      <c r="B13" s="3" t="s">
+        <v>7</v>
       </c>
       <c r="C13" s="1">
-        <v>1.97028826221731E-4</v>
+        <v>3.2791453922484702E-4</v>
       </c>
       <c r="D13" s="1">
-        <v>5.8891870032100595E-4</v>
+        <v>1.91218155012373E-4</v>
       </c>
       <c r="E13" s="1">
-        <v>0.33456031556534899</v>
-      </c>
-      <c r="F13" s="1">
-        <v>0.73962183969531003</v>
+        <v>1.7148713687967001</v>
+      </c>
+      <c r="F13" s="3">
+        <v>9.3739580007072595E-2</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
@@ -1850,22 +1850,22 @@
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" s="8" t="s">
-        <v>13</v>
-      </c>
-      <c r="B15" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="C15" s="1">
-        <v>-9.2289269036274994E-3</v>
-      </c>
-      <c r="D15" s="1">
-        <v>2.0219582698712199E-3</v>
+        <v>6</v>
+      </c>
+      <c r="B15" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="C15" s="2">
+        <v>-3.5825154663033903E-5</v>
+      </c>
+      <c r="D15" s="2">
+        <v>1.8927460038076501E-5</v>
       </c>
       <c r="E15" s="1">
-        <v>-4.5643508281777203</v>
-      </c>
-      <c r="F15" s="5">
-        <v>4.32123185112372E-5</v>
+        <v>-1.89276081370476</v>
+      </c>
+      <c r="F15" s="3">
+        <v>6.5294653231981498E-2</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
@@ -1873,35 +1873,35 @@
       <c r="B16" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="C16" s="1">
-        <v>-7.3045528780302498E-3</v>
-      </c>
-      <c r="D16" s="1">
-        <v>1.3201702736387801E-2</v>
+      <c r="C16" s="2">
+        <v>-5.8390208894141502E-5</v>
+      </c>
+      <c r="D16" s="2">
+        <v>4.0125816043901601E-5</v>
       </c>
       <c r="E16" s="1">
-        <v>-0.55330384450308201</v>
+        <v>-1.4551781035495199</v>
       </c>
       <c r="F16" s="1">
-        <v>0.58298890967638495</v>
+        <v>0.15305398014178601</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17" s="8"/>
-      <c r="B17" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="C17" s="1">
-        <v>5.8817294904817104E-3</v>
-      </c>
-      <c r="D17" s="1">
-        <v>6.2272802303673597E-3</v>
+      <c r="B17" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C17" s="2">
+        <v>1.3575622868601501E-5</v>
+      </c>
+      <c r="D17" s="2">
+        <v>6.1456258488287402E-6</v>
       </c>
       <c r="E17" s="1">
-        <v>0.94451016702274404</v>
-      </c>
-      <c r="F17" s="1">
-        <v>0.35031110487931999</v>
+        <v>2.2089894833394101</v>
+      </c>
+      <c r="F17" s="4">
+        <v>3.2684032924149502E-2</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.25">
@@ -1909,73 +1909,73 @@
       <c r="B18" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="C18" s="1">
-        <v>5.1637448869641103E-3</v>
-      </c>
-      <c r="D18" s="1">
-        <v>9.3498634940876301E-3</v>
+      <c r="C18" s="2">
+        <v>-3.0176903192067899E-5</v>
+      </c>
+      <c r="D18" s="2">
+        <v>2.84183722426402E-5</v>
       </c>
       <c r="E18" s="1">
-        <v>0.552280243474078</v>
+        <v>-1.06188007301801</v>
       </c>
       <c r="F18" s="1">
-        <v>0.58368360811750397</v>
+        <v>0.29435811396760603</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A19" s="8" t="s">
-        <v>14</v>
-      </c>
-      <c r="B19" s="1" t="s">
-        <v>7</v>
+        <v>11</v>
+      </c>
+      <c r="B19" s="4" t="s">
+        <v>9</v>
       </c>
       <c r="C19" s="1">
-        <v>-5.8861885046492099E-4</v>
+        <v>2.15160279809898E-3</v>
       </c>
       <c r="D19" s="1">
-        <v>1.4346376785910201E-3</v>
+        <v>9.6063412902913897E-4</v>
       </c>
       <c r="E19" s="1">
-        <v>-0.41029094610355599</v>
-      </c>
-      <c r="F19" s="1">
-        <v>0.68367806403607001</v>
+        <v>2.2397734299462102</v>
+      </c>
+      <c r="F19" s="4">
+        <v>3.0456337762944499E-2</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20" s="8"/>
-      <c r="B20" s="1" t="s">
+      <c r="B20" s="4" t="s">
         <v>8</v>
       </c>
       <c r="C20" s="1">
-        <v>4.0722147842239403E-3</v>
+        <v>-7.5561135023714298E-3</v>
       </c>
       <c r="D20" s="1">
-        <v>9.3669886512477308E-3</v>
+        <v>2.03652409089086E-3</v>
       </c>
       <c r="E20" s="1">
-        <v>0.43474108230946801</v>
-      </c>
-      <c r="F20" s="1">
-        <v>0.66597601145868301</v>
+        <v>-3.7102991003981001</v>
+      </c>
+      <c r="F20" s="4">
+        <v>6.0210191906117001E-4</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A21" s="8"/>
-      <c r="B21" s="4" t="s">
-        <v>9</v>
+      <c r="B21" s="3" t="s">
+        <v>7</v>
       </c>
       <c r="C21" s="1">
-        <v>1.8270517684183099E-2</v>
+        <v>-5.5751340316831095E-4</v>
       </c>
       <c r="D21" s="1">
-        <v>4.4184348345621396E-3</v>
+        <v>3.1191178968292902E-4</v>
       </c>
       <c r="E21" s="1">
-        <v>4.1350655533643597</v>
-      </c>
-      <c r="F21" s="4">
-        <v>1.6614380889968299E-4</v>
+        <v>-1.7874072786252999</v>
+      </c>
+      <c r="F21" s="3">
+        <v>8.1089298193969594E-2</v>
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.25">
@@ -1983,73 +1983,73 @@
       <c r="B22" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="C22" s="1">
-        <v>-4.5367957521503504E-3</v>
+      <c r="C22" s="2">
+        <v>3.5716593827619803E-5</v>
       </c>
       <c r="D22" s="1">
-        <v>6.6339976735302003E-3</v>
+        <v>1.4423307835713601E-3</v>
       </c>
       <c r="E22" s="1">
-        <v>-0.68387056725272399</v>
+        <v>2.47631085978639E-2</v>
       </c>
       <c r="F22" s="1">
-        <v>0.49781289740463303</v>
+        <v>0.98036120027870799</v>
       </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A23" s="8" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="C23" s="1">
-        <v>-5.8392474847676103E-4</v>
+        <v>5.8817294904817104E-3</v>
       </c>
       <c r="D23" s="1">
-        <v>1.3895256343106001E-3</v>
+        <v>6.2272802303673597E-3</v>
       </c>
       <c r="E23" s="1">
-        <v>-0.42023316019389001</v>
+        <v>0.94451016702274404</v>
       </c>
       <c r="F23" s="1">
-        <v>0.67645737999211397</v>
+        <v>0.35031110487931999</v>
       </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A24" s="8"/>
-      <c r="B24" s="3" t="s">
+      <c r="B24" s="1" t="s">
         <v>8</v>
       </c>
       <c r="C24" s="1">
-        <v>1.59394994363261E-2</v>
+        <v>-7.3045528780302498E-3</v>
       </c>
       <c r="D24" s="1">
-        <v>9.0724445910189706E-3</v>
+        <v>1.3201702736387801E-2</v>
       </c>
       <c r="E24" s="1">
-        <v>1.75691339598866</v>
-      </c>
-      <c r="F24" s="3">
-        <v>8.6221150816636699E-2</v>
+        <v>-0.55330384450308201</v>
+      </c>
+      <c r="F24" s="1">
+        <v>0.58298890967638495</v>
       </c>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A25" s="8"/>
       <c r="B25" s="4" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="C25" s="1">
-        <v>1.5654496005932599E-2</v>
+        <v>-9.2289269036274994E-3</v>
       </c>
       <c r="D25" s="1">
-        <v>4.2794975747358702E-3</v>
+        <v>2.0219582698712199E-3</v>
       </c>
       <c r="E25" s="1">
-        <v>3.6580219365818301</v>
-      </c>
-      <c r="F25" s="4">
-        <v>7.0287164406071902E-4</v>
+        <v>-4.5643508281777203</v>
+      </c>
+      <c r="F25" s="5">
+        <v>4.32123185112372E-5</v>
       </c>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.25">
@@ -2058,36 +2058,36 @@
         <v>10</v>
       </c>
       <c r="C26" s="1">
-        <v>2.5105742368774402E-3</v>
+        <v>5.1637448869641103E-3</v>
       </c>
       <c r="D26" s="1">
-        <v>6.4253922526141096E-3</v>
+        <v>9.3498634940876301E-3</v>
       </c>
       <c r="E26" s="1">
-        <v>0.39072699971834901</v>
+        <v>0.552280243474078</v>
       </c>
       <c r="F26" s="1">
-        <v>0.69797399323822196</v>
+        <v>0.58368360811750397</v>
       </c>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A27" s="8" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="B27" s="4" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="C27" s="1">
-        <v>3.6091968136373401E-4</v>
-      </c>
-      <c r="D27" s="2">
-        <v>8.7899019274630306E-5</v>
+        <v>1.8270517684183099E-2</v>
+      </c>
+      <c r="D27" s="1">
+        <v>4.4184348345621396E-3</v>
       </c>
       <c r="E27" s="1">
-        <v>4.1060717666949396</v>
+        <v>4.1350655533643597</v>
       </c>
       <c r="F27" s="4">
-        <v>1.8169073902427901E-4</v>
+        <v>1.6614380889968299E-4</v>
       </c>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.25">
@@ -2096,34 +2096,34 @@
         <v>8</v>
       </c>
       <c r="C28" s="1">
-        <v>-2.7141891938760603E-4</v>
+        <v>4.0722147842239403E-3</v>
       </c>
       <c r="D28" s="1">
-        <v>5.7390735534695305E-4</v>
+        <v>9.3669886512477308E-3</v>
       </c>
       <c r="E28" s="1">
-        <v>-0.47293159228377701</v>
+        <v>0.43474108230946801</v>
       </c>
       <c r="F28" s="1">
-        <v>0.63871063739713796</v>
+        <v>0.66597601145868301</v>
       </c>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A29" s="8"/>
       <c r="B29" s="1" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="C29" s="1">
-        <v>-3.64146958916518E-4</v>
+        <v>-5.8861885046492099E-4</v>
       </c>
       <c r="D29" s="1">
-        <v>2.7071371014617701E-4</v>
+        <v>1.4346376785910201E-3</v>
       </c>
       <c r="E29" s="1">
-        <v>-1.34513674508724</v>
+        <v>-0.41029094610355599</v>
       </c>
       <c r="F29" s="1">
-        <v>0.185799557133072</v>
+        <v>0.68367806403607001</v>
       </c>
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.25">
@@ -2131,73 +2131,73 @@
       <c r="B30" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="C30" s="2">
-        <v>-6.1139804463442406E-5</v>
+      <c r="C30" s="1">
+        <v>-4.5367957521503504E-3</v>
       </c>
       <c r="D30" s="1">
-        <v>4.0645934376000399E-4</v>
+        <v>6.6339976735302003E-3</v>
       </c>
       <c r="E30" s="1">
-        <v>-0.150420467390074</v>
+        <v>-0.68387056725272399</v>
       </c>
       <c r="F30" s="1">
-        <v>0.88115298754952798</v>
+        <v>0.49781289740463303</v>
       </c>
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A31" s="8" t="s">
-        <v>17</v>
-      </c>
-      <c r="B31" s="1" t="s">
-        <v>7</v>
+        <v>15</v>
+      </c>
+      <c r="B31" s="4" t="s">
+        <v>9</v>
       </c>
       <c r="C31" s="1">
-        <v>1.6039099443968701E-4</v>
+        <v>1.5654496005932599E-2</v>
       </c>
       <c r="D31" s="1">
-        <v>1.66294157162633E-4</v>
+        <v>4.2794975747358702E-3</v>
       </c>
       <c r="E31" s="1">
-        <v>0.96450168289934102</v>
-      </c>
-      <c r="F31" s="1">
-        <v>0.34031531873463899</v>
+        <v>3.6580219365818301</v>
+      </c>
+      <c r="F31" s="4">
+        <v>7.0287164406071902E-4</v>
       </c>
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A32" s="8"/>
-      <c r="B32" s="1" t="s">
+      <c r="B32" s="3" t="s">
         <v>8</v>
       </c>
       <c r="C32" s="1">
-        <v>5.7953254205743605E-4</v>
+        <v>1.59394994363261E-2</v>
       </c>
       <c r="D32" s="1">
-        <v>1.08576228420335E-3</v>
+        <v>9.0724445910189706E-3</v>
       </c>
       <c r="E32" s="1">
-        <v>0.53375637604013104</v>
-      </c>
-      <c r="F32" s="1">
-        <v>0.59632390024812099</v>
+        <v>1.75691339598866</v>
+      </c>
+      <c r="F32" s="3">
+        <v>8.6221150816636699E-2</v>
       </c>
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A33" s="8"/>
-      <c r="B33" s="4" t="s">
-        <v>9</v>
+      <c r="B33" s="1" t="s">
+        <v>7</v>
       </c>
       <c r="C33" s="1">
-        <v>1.4546674291028201E-3</v>
+        <v>-5.8392474847676103E-4</v>
       </c>
       <c r="D33" s="1">
-        <v>5.1215711657116403E-4</v>
+        <v>1.3895256343106001E-3</v>
       </c>
       <c r="E33" s="1">
-        <v>2.8402757318724001</v>
-      </c>
-      <c r="F33" s="4">
-        <v>6.9216450943544302E-3</v>
+        <v>-0.42023316019389001</v>
+      </c>
+      <c r="F33" s="1">
+        <v>0.67645737999211397</v>
       </c>
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.25">
@@ -2206,28 +2206,28 @@
         <v>10</v>
       </c>
       <c r="C34" s="1">
-        <v>-7.5215013217949395E-4</v>
+        <v>2.5105742368774402E-3</v>
       </c>
       <c r="D34" s="1">
-        <v>7.6897119614342802E-4</v>
+        <v>6.4253922526141096E-3</v>
       </c>
       <c r="E34" s="1">
-        <v>-0.97812523531662099</v>
+        <v>0.39072699971834901</v>
       </c>
       <c r="F34" s="1">
-        <v>0.33361305843751698</v>
+        <v>0.69797399323822196</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="9">
+    <mergeCell ref="A19:A22"/>
+    <mergeCell ref="A15:A18"/>
+    <mergeCell ref="A1:F1"/>
     <mergeCell ref="A7:A10"/>
     <mergeCell ref="A3:A6"/>
-    <mergeCell ref="A1:F1"/>
     <mergeCell ref="A31:A34"/>
     <mergeCell ref="A27:A30"/>
     <mergeCell ref="A23:A26"/>
-    <mergeCell ref="A19:A22"/>
-    <mergeCell ref="A15:A18"/>
     <mergeCell ref="A11:A14"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
community metrics and FD analysis and figures updated with last species removed due to 0 germination. No significant changes to the results
</commit_message>
<xml_diff>
--- a/results/CM vs microclimatic gradients.xlsx
+++ b/results/CM vs microclimatic gradients.xlsx
@@ -987,16 +987,16 @@
         <v>9</v>
       </c>
       <c r="C3" s="1">
-        <v>-3.6072578934203299E-3</v>
+        <v>-3.1639373829148599E-3</v>
       </c>
       <c r="D3" s="1">
-        <v>1.2690195160271101E-3</v>
+        <v>1.2367227543779299E-3</v>
       </c>
       <c r="E3" s="1">
-        <v>-2.8425550969566702</v>
+        <v>-2.5583239021961002</v>
       </c>
       <c r="F3" s="4">
-        <v>6.6521005502137602E-3</v>
+        <v>1.4122840032780901E-2</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
@@ -1005,16 +1005,16 @@
         <v>8</v>
       </c>
       <c r="C4" s="1">
-        <v>-1.4862568015520301E-4</v>
+        <v>-1.0941471184459199E-3</v>
       </c>
       <c r="D4" s="1">
-        <v>1.4049986044080099E-3</v>
+        <v>1.3248731769758E-3</v>
       </c>
       <c r="E4" s="1">
-        <v>-0.105783507320868</v>
+        <v>-0.82585045682897296</v>
       </c>
       <c r="F4" s="1">
-        <v>0.91621408320581599</v>
+        <v>0.41344764379413201</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
@@ -1023,34 +1023,34 @@
         <v>7</v>
       </c>
       <c r="C5" s="2">
-        <v>5.2599606029830298E-5</v>
+        <v>-8.2451333541634105E-5</v>
       </c>
       <c r="D5" s="1">
-        <v>1.10671708895486E-4</v>
+        <v>1.05640675692154E-4</v>
       </c>
       <c r="E5" s="1">
-        <v>0.475275990176528</v>
+        <v>-0.78048850976591699</v>
       </c>
       <c r="F5" s="1">
-        <v>0.63683937849943295</v>
+        <v>0.43937894332400401</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" s="8"/>
-      <c r="B6" s="3" t="s">
+      <c r="B6" s="1" t="s">
         <v>10</v>
       </c>
       <c r="C6" s="1">
-        <v>1.50116471133251E-3</v>
+        <v>1.1473003586561399E-3</v>
       </c>
       <c r="D6" s="1">
-        <v>8.0749822162049705E-4</v>
+        <v>7.7408646332860899E-4</v>
       </c>
       <c r="E6" s="1">
-        <v>1.85903160049066</v>
-      </c>
-      <c r="F6" s="3">
-        <v>6.9426541584144894E-2</v>
+        <v>1.4821346361266801</v>
+      </c>
+      <c r="F6" s="1">
+        <v>0.14559651443604699</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
@@ -1061,16 +1061,16 @@
         <v>9</v>
       </c>
       <c r="C7" s="1">
-        <v>-9.7186664867520405E-3</v>
+        <v>-8.2949162830517308E-3</v>
       </c>
       <c r="D7" s="1">
-        <v>3.37966265215105E-3</v>
+        <v>3.2424925026586799E-3</v>
       </c>
       <c r="E7" s="1">
-        <v>-2.8756321227997201</v>
+        <v>-2.5581913531797902</v>
       </c>
       <c r="F7" s="4">
-        <v>6.0899396888603203E-3</v>
+        <v>1.4127497639785699E-2</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
@@ -1079,34 +1079,34 @@
         <v>8</v>
       </c>
       <c r="C8" s="1">
-        <v>-2.96547411479808E-3</v>
+        <v>-2.4654252839035199E-3</v>
       </c>
       <c r="D8" s="1">
-        <v>3.7418032186832401E-3</v>
+        <v>3.47360904302147E-3</v>
       </c>
       <c r="E8" s="1">
-        <v>-0.792525405930256</v>
+        <v>-0.70975900090328004</v>
       </c>
       <c r="F8" s="1">
-        <v>0.43212287909522301</v>
+        <v>0.48168492932136803</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" s="10"/>
-      <c r="B9" s="4" t="s">
+      <c r="B9" s="3" t="s">
         <v>7</v>
       </c>
       <c r="C9" s="1">
-        <v>6.1703022608801503E-4</v>
+        <v>5.0352839348548296E-4</v>
       </c>
       <c r="D9" s="1">
-        <v>2.9474175651355102E-4</v>
+        <v>2.76973232436322E-4</v>
       </c>
       <c r="E9" s="1">
-        <v>2.0934605038212402</v>
-      </c>
-      <c r="F9" s="4">
-        <v>4.1849565675452997E-2</v>
+        <v>1.8179677113789301</v>
+      </c>
+      <c r="F9" s="3">
+        <v>7.60401242360048E-2</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
@@ -1115,16 +1115,16 @@
         <v>10</v>
       </c>
       <c r="C10" s="1">
-        <v>2.6048141438072699E-3</v>
+        <v>1.94946263119698E-3</v>
       </c>
       <c r="D10" s="1">
-        <v>2.1505355487621098E-3</v>
+        <v>2.0295329287566099E-3</v>
       </c>
       <c r="E10" s="1">
-        <v>1.2112397515617199</v>
+        <v>0.96054742624516698</v>
       </c>
       <c r="F10" s="1">
-        <v>0.23198952469817799</v>
+        <v>0.34215017207589499</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
@@ -1135,16 +1135,16 @@
         <v>9</v>
       </c>
       <c r="C11" s="1">
-        <v>-9.6861009576420208E-3</v>
+        <v>-7.3199717780581403E-3</v>
       </c>
       <c r="D11" s="1">
-        <v>2.19958355944536E-3</v>
+        <v>1.91879139414312E-3</v>
       </c>
       <c r="E11" s="1">
-        <v>-4.4036067263952603</v>
-      </c>
-      <c r="F11" s="5">
-        <v>6.2977067874974701E-5</v>
+        <v>-3.8148867044127202</v>
+      </c>
+      <c r="F11" s="4">
+        <v>4.3079157074682098E-4</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
@@ -1153,16 +1153,16 @@
         <v>8</v>
       </c>
       <c r="C12" s="1">
-        <v>2.8114732251873799E-4</v>
+        <v>-7.2670392364368702E-4</v>
       </c>
       <c r="D12" s="1">
-        <v>2.4352752595756802E-3</v>
+        <v>2.0555579181454598E-3</v>
       </c>
       <c r="E12" s="1">
-        <v>0.115447862172149</v>
+        <v>-0.353531232191855</v>
       </c>
       <c r="F12" s="1">
-        <v>0.90859264839932996</v>
+        <v>0.72541770992343202</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
@@ -1170,17 +1170,17 @@
       <c r="B13" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="C13" s="1">
-        <v>2.3166489008347299E-4</v>
+      <c r="C13" s="2">
+        <v>-1.02130892504796E-5</v>
       </c>
       <c r="D13" s="1">
-        <v>1.91826578163541E-4</v>
+        <v>1.6390287853281101E-4</v>
       </c>
       <c r="E13" s="1">
-        <v>1.20767879144447</v>
+        <v>-6.2311835776789497E-2</v>
       </c>
       <c r="F13" s="1">
-        <v>0.233343635342591</v>
+        <v>0.95060325051934902</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
@@ -1189,36 +1189,36 @@
         <v>10</v>
       </c>
       <c r="C14" s="1">
-        <v>1.4460403611902099E-3</v>
+        <v>1.11173519179463E-4</v>
       </c>
       <c r="D14" s="1">
-        <v>1.3996315975647101E-3</v>
+        <v>1.2010051880259299E-3</v>
       </c>
       <c r="E14" s="1">
-        <v>1.0331578421823699</v>
+        <v>9.2567059899380702E-2</v>
       </c>
       <c r="F14" s="1">
-        <v>0.30693143969161801</v>
+        <v>0.92667745079887498</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" s="8" t="s">
         <v>6</v>
       </c>
-      <c r="B15" s="3" t="s">
+      <c r="B15" s="1" t="s">
         <v>9</v>
       </c>
       <c r="C15" s="1">
-        <v>-2.4835389120634401E-4</v>
+        <v>-1.57738468001018E-4</v>
       </c>
       <c r="D15" s="1">
-        <v>1.23875119163699E-4</v>
+        <v>1.1298801668997701E-4</v>
       </c>
       <c r="E15" s="1">
-        <v>-2.0048730760706501</v>
-      </c>
-      <c r="F15" s="3">
-        <v>5.0882349685987899E-2</v>
+        <v>-1.3960636943812399</v>
+      </c>
+      <c r="F15" s="1">
+        <v>0.16986171773994699</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
@@ -1227,16 +1227,16 @@
         <v>8</v>
       </c>
       <c r="C16" s="2">
-        <v>2.0349472277592401E-5</v>
+        <v>4.3898833434660098E-5</v>
       </c>
       <c r="D16" s="1">
-        <v>1.3714869420665001E-4</v>
+        <v>1.21041512418473E-4</v>
       </c>
       <c r="E16" s="1">
-        <v>0.148375253554588</v>
+        <v>0.36267585027267502</v>
       </c>
       <c r="F16" s="1">
-        <v>0.88269515722479497</v>
+        <v>0.71862367443616804</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.25">
@@ -1245,16 +1245,16 @@
         <v>7</v>
       </c>
       <c r="C17" s="2">
-        <v>1.8233142963540399E-5</v>
+        <v>1.5067436244838899E-5</v>
       </c>
       <c r="D17" s="2">
-        <v>1.08031995996393E-5</v>
+        <v>9.6514197591920197E-6</v>
       </c>
       <c r="E17" s="1">
-        <v>1.6877539654223499</v>
+        <v>1.56116267044428</v>
       </c>
       <c r="F17" s="1">
-        <v>9.8228581389421102E-2</v>
+        <v>0.125815909975315</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.25">
@@ -1262,17 +1262,17 @@
       <c r="B18" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="C18" s="1">
-        <v>1.1983767405981699E-4</v>
+      <c r="C18" s="2">
+        <v>9.2822725670461004E-5</v>
       </c>
       <c r="D18" s="2">
-        <v>7.8823798345412999E-5</v>
+        <v>7.0721181387214997E-5</v>
       </c>
       <c r="E18" s="1">
-        <v>1.520323513651</v>
+        <v>1.3125166159518</v>
       </c>
       <c r="F18" s="1">
-        <v>0.13527418652671999</v>
+        <v>0.196308657605195</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.25">
@@ -1282,17 +1282,17 @@
       <c r="B19" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="C19" s="1">
-        <v>1.5479634490939999E-3</v>
+      <c r="C19" s="2">
+        <v>2.7477501223953501E-5</v>
       </c>
       <c r="D19" s="1">
-        <v>7.3982850709574796E-3</v>
+        <v>6.7749375145306897E-4</v>
       </c>
       <c r="E19" s="1">
-        <v>0.209232738972258</v>
+        <v>4.05575714388813E-2</v>
       </c>
       <c r="F19" s="1">
-        <v>0.83519040955672696</v>
+        <v>0.967836341228964</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.25">
@@ -1301,34 +1301,34 @@
         <v>8</v>
       </c>
       <c r="C20" s="1">
-        <v>-2.0343295228709299E-2</v>
+        <v>-2.5600486619732602E-3</v>
       </c>
       <c r="D20" s="1">
-        <v>8.1910325794278798E-3</v>
+        <v>7.2578376656485502E-4</v>
       </c>
       <c r="E20" s="1">
-        <v>-2.4836057031200598</v>
+        <v>-3.5272884017370698</v>
       </c>
       <c r="F20" s="4">
-        <v>1.6711393192260102E-2</v>
+        <v>1.01276113190216E-3</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A21" s="8"/>
-      <c r="B21" s="1" t="s">
+      <c r="B21" s="4" t="s">
         <v>7</v>
       </c>
       <c r="C21" s="1">
-        <v>-1.1152605499439199E-3</v>
-      </c>
-      <c r="D21" s="1">
-        <v>6.4520745454109505E-4</v>
+        <v>-1.5570885383056499E-4</v>
+      </c>
+      <c r="D21" s="2">
+        <v>5.7871416554241799E-5</v>
       </c>
       <c r="E21" s="1">
-        <v>-1.72853016823427</v>
-      </c>
-      <c r="F21" s="1">
-        <v>9.0600955728569299E-2</v>
+        <v>-2.69060035336482</v>
+      </c>
+      <c r="F21" s="4">
+        <v>1.01158333143496E-2</v>
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.25">
@@ -1337,16 +1337,16 @@
         <v>10</v>
       </c>
       <c r="C22" s="1">
-        <v>-6.6518676371898899E-3</v>
+        <v>-6.4081441799058395E-4</v>
       </c>
       <c r="D22" s="1">
-        <v>4.7076518228361302E-3</v>
+        <v>4.2405522186201498E-4</v>
       </c>
       <c r="E22" s="1">
-        <v>-1.4129905709939401</v>
+        <v>-1.5111579458372999</v>
       </c>
       <c r="F22" s="1">
-        <v>0.164389493719657</v>
+        <v>0.13806294776920799</v>
       </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.25">
@@ -1357,16 +1357,16 @@
         <v>9</v>
       </c>
       <c r="C23" s="1">
-        <v>2.9569378756749299E-2</v>
+        <v>4.3135270409365399E-3</v>
       </c>
       <c r="D23" s="1">
-        <v>2.4952471535037001E-2</v>
+        <v>2.2605787562698699E-2</v>
       </c>
       <c r="E23" s="1">
-        <v>1.18502805284156</v>
+        <v>0.19081516310691099</v>
       </c>
       <c r="F23" s="1">
-        <v>0.24209258446117399</v>
+        <v>0.84956849186100003</v>
       </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.25">
@@ -1375,16 +1375,16 @@
         <v>8</v>
       </c>
       <c r="C24" s="1">
-        <v>2.9038975186392601E-2</v>
+        <v>3.2674067292850099E-2</v>
       </c>
       <c r="D24" s="1">
-        <v>2.76262005749238E-2</v>
+        <v>2.4217070058921299E-2</v>
       </c>
       <c r="E24" s="1">
-        <v>1.0511389399218101</v>
+        <v>1.34921636735379</v>
       </c>
       <c r="F24" s="1">
-        <v>0.29868563930830799</v>
+        <v>0.18432937712376299</v>
       </c>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.25">
@@ -1393,16 +1393,16 @@
         <v>7</v>
       </c>
       <c r="C25" s="1">
-        <v>-1.7997596633955601E-4</v>
+        <v>1.98269004059539E-4</v>
       </c>
       <c r="D25" s="1">
-        <v>2.1761152063240002E-3</v>
+        <v>1.9309830471082299E-3</v>
       </c>
       <c r="E25" s="1">
-        <v>-8.2705164605499204E-2</v>
+        <v>0.10267775491683299</v>
       </c>
       <c r="F25" s="1">
-        <v>0.93444482661378703</v>
+        <v>0.91869608668671299</v>
       </c>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.25">
@@ -1411,36 +1411,36 @@
         <v>10</v>
       </c>
       <c r="C26" s="1">
-        <v>-6.3905265837868796E-3</v>
+        <v>1.6918077207999001E-3</v>
       </c>
       <c r="D26" s="1">
-        <v>1.5877672592978499E-2</v>
+        <v>1.41493589272311E-2</v>
       </c>
       <c r="E26" s="1">
-        <v>-0.40248509637444702</v>
+        <v>0.119567800173896</v>
       </c>
       <c r="F26" s="1">
-        <v>0.68919137950349796</v>
+        <v>0.90538242349200604</v>
       </c>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A27" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="B27" s="3" t="s">
+      <c r="B27" s="1" t="s">
         <v>9</v>
       </c>
       <c r="C27" s="1">
-        <v>4.4088729294911803E-2</v>
+        <v>2.99095423901602E-2</v>
       </c>
       <c r="D27" s="1">
-        <v>2.3256853979988699E-2</v>
+        <v>2.2586166157614E-2</v>
       </c>
       <c r="E27" s="1">
-        <v>1.89573058044944</v>
-      </c>
-      <c r="F27" s="3">
-        <v>6.4288284198534898E-2</v>
+        <v>1.32424166994262</v>
+      </c>
+      <c r="F27" s="1">
+        <v>0.19241885737343001</v>
       </c>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.25">
@@ -1449,16 +1449,16 @@
         <v>8</v>
       </c>
       <c r="C28" s="1">
-        <v>-5.7096452452447301E-3</v>
+        <v>3.5383422499573598E-3</v>
       </c>
       <c r="D28" s="1">
-        <v>2.5748892725544901E-2</v>
+        <v>2.4196050090461E-2</v>
       </c>
       <c r="E28" s="1">
-        <v>-0.22174333110566499</v>
+        <v>0.14623635827867301</v>
       </c>
       <c r="F28" s="1">
-        <v>0.82549518635725805</v>
+        <v>0.88441823350904503</v>
       </c>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.25">
@@ -1467,16 +1467,16 @@
         <v>7</v>
       </c>
       <c r="C29" s="1">
-        <v>6.1875044666251204E-4</v>
+        <v>5.6283393360731699E-4</v>
       </c>
       <c r="D29" s="1">
-        <v>2.0282397086816301E-3</v>
+        <v>1.92930698957324E-3</v>
       </c>
       <c r="E29" s="1">
-        <v>0.30506771167827301</v>
+        <v>0.29172855157271599</v>
       </c>
       <c r="F29" s="1">
-        <v>0.76169070210021295</v>
+        <v>0.77189698592883504</v>
       </c>
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.25">
@@ -1485,16 +1485,16 @@
         <v>10</v>
       </c>
       <c r="C30" s="1">
-        <v>-2.7282682462299803E-4</v>
+        <v>-3.6103141714002801E-3</v>
       </c>
       <c r="D30" s="1">
-        <v>1.47987229448781E-2</v>
+        <v>1.41370775456411E-2</v>
       </c>
       <c r="E30" s="1">
-        <v>-1.8435835689283201E-2</v>
+        <v>-0.255379102204433</v>
       </c>
       <c r="F30" s="1">
-        <v>0.98537089879256601</v>
+        <v>0.79964792899491699</v>
       </c>
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.25">
@@ -1505,16 +1505,16 @@
         <v>9</v>
       </c>
       <c r="C31" s="1">
-        <v>5.8825892885889103E-2</v>
+        <v>5.2974170081300703E-2</v>
       </c>
       <c r="D31" s="1">
-        <v>1.47625055825771E-2</v>
+        <v>1.5296042864919999E-2</v>
       </c>
       <c r="E31" s="1">
-        <v>3.9848176555690098</v>
+        <v>3.46325978222719</v>
       </c>
       <c r="F31" s="4">
-        <v>2.3896406994294701E-4</v>
+        <v>1.2202745969677299E-3</v>
       </c>
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.25">
@@ -1523,16 +1523,16 @@
         <v>8</v>
       </c>
       <c r="C32" s="1">
-        <v>-1.4775078079508E-2</v>
+        <v>-1.62357606830522E-2</v>
       </c>
       <c r="D32" s="1">
-        <v>1.6344350484081199E-2</v>
+        <v>1.63863055271413E-2</v>
       </c>
       <c r="E32" s="1">
-        <v>-0.90398686040772402</v>
+        <v>-0.99081276472968605</v>
       </c>
       <c r="F32" s="1">
-        <v>0.37071241321783299</v>
+        <v>0.327319965428154</v>
       </c>
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.25">
@@ -1541,47 +1541,47 @@
         <v>7</v>
       </c>
       <c r="C33" s="1">
-        <v>-7.2151906794048603E-4</v>
+        <v>-1.1828483567966599E-3</v>
       </c>
       <c r="D33" s="1">
-        <v>1.2874441249869999E-3</v>
+        <v>1.30658573067097E-3</v>
       </c>
       <c r="E33" s="1">
-        <v>-0.56042748103555196</v>
+        <v>-0.90529716422758599</v>
       </c>
       <c r="F33" s="1">
-        <v>0.57790738199043301</v>
+        <v>0.37035269499112</v>
       </c>
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A34" s="8"/>
-      <c r="B34" s="1" t="s">
+      <c r="B34" s="3" t="s">
         <v>10</v>
       </c>
       <c r="C34" s="1">
-        <v>-1.37319352158409E-2</v>
+        <v>-1.91295126674411E-2</v>
       </c>
       <c r="D34" s="1">
-        <v>9.3936278000778892E-3</v>
+        <v>9.5740615124239696E-3</v>
       </c>
       <c r="E34" s="1">
-        <v>-1.4618351405968</v>
-      </c>
-      <c r="F34" s="1">
-        <v>0.150584814092001</v>
+        <v>-1.99805616901639</v>
+      </c>
+      <c r="F34" s="3">
+        <v>5.2060315386044498E-2</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="9">
+    <mergeCell ref="A31:A34"/>
+    <mergeCell ref="A27:A30"/>
+    <mergeCell ref="A23:A26"/>
+    <mergeCell ref="A11:A14"/>
     <mergeCell ref="A19:A22"/>
     <mergeCell ref="A15:A18"/>
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="A7:A10"/>
     <mergeCell ref="A3:A6"/>
-    <mergeCell ref="A31:A34"/>
-    <mergeCell ref="A27:A30"/>
-    <mergeCell ref="A23:A26"/>
-    <mergeCell ref="A11:A14"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
@@ -1634,16 +1634,16 @@
         <v>9</v>
       </c>
       <c r="C3" s="1">
-        <v>-3.64146958916518E-4</v>
+        <v>-3.5451294042417101E-4</v>
       </c>
       <c r="D3" s="1">
-        <v>2.7071371014617701E-4</v>
+        <v>2.7045603053708699E-4</v>
       </c>
       <c r="E3" s="1">
-        <v>-1.34513674508724</v>
+        <v>-1.31079695180085</v>
       </c>
       <c r="F3" s="1">
-        <v>0.185799557133072</v>
+        <v>0.197048754373924</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
@@ -1652,16 +1652,16 @@
         <v>8</v>
       </c>
       <c r="C4" s="1">
-        <v>-2.7141891938760603E-4</v>
+        <v>-2.8778074405096002E-4</v>
       </c>
       <c r="D4" s="1">
-        <v>5.7390735534695305E-4</v>
+        <v>5.7336108001091596E-4</v>
       </c>
       <c r="E4" s="1">
-        <v>-0.47293159228377701</v>
+        <v>-0.50191886768017302</v>
       </c>
       <c r="F4" s="1">
-        <v>0.63871063739713796</v>
+        <v>0.61834579898509201</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
@@ -1670,16 +1670,16 @@
         <v>7</v>
       </c>
       <c r="C5" s="1">
-        <v>3.6091968136373401E-4</v>
+        <v>3.5567938949130701E-4</v>
       </c>
       <c r="D5" s="2">
-        <v>8.7899019274630306E-5</v>
+        <v>8.7815352345039198E-5</v>
       </c>
       <c r="E5" s="1">
-        <v>4.1060717666949396</v>
+        <v>4.0503098831032602</v>
       </c>
       <c r="F5" s="4">
-        <v>1.8169073902427901E-4</v>
+        <v>2.1566881395634199E-4</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
@@ -1688,16 +1688,16 @@
         <v>10</v>
       </c>
       <c r="C6" s="2">
-        <v>-6.1139804463442406E-5</v>
+        <v>-3.22947514131102E-5</v>
       </c>
       <c r="D6" s="1">
-        <v>4.0645934376000399E-4</v>
+        <v>4.0607245428641702E-4</v>
       </c>
       <c r="E6" s="1">
-        <v>-0.150420467390074</v>
+        <v>-7.9529529945243801E-2</v>
       </c>
       <c r="F6" s="1">
-        <v>0.88115298754952798</v>
+        <v>0.93698917829126904</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
@@ -1708,16 +1708,16 @@
         <v>9</v>
       </c>
       <c r="C7" s="1">
-        <v>1.4546674291028201E-3</v>
+        <v>1.5212248193409101E-3</v>
       </c>
       <c r="D7" s="1">
-        <v>5.1215711657116403E-4</v>
+        <v>5.0548939164991901E-4</v>
       </c>
       <c r="E7" s="1">
-        <v>2.8402757318724001</v>
+        <v>3.00940997866569</v>
       </c>
       <c r="F7" s="4">
-        <v>6.9216450943544302E-3</v>
+        <v>4.4127755964004801E-3</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
@@ -1726,16 +1726,16 @@
         <v>8</v>
       </c>
       <c r="C8" s="1">
-        <v>5.7953254205743605E-4</v>
+        <v>4.78722634661545E-4</v>
       </c>
       <c r="D8" s="1">
-        <v>1.08576228420335E-3</v>
+        <v>1.0716268480126E-3</v>
       </c>
       <c r="E8" s="1">
-        <v>0.53375637604013104</v>
+        <v>0.44672512222828897</v>
       </c>
       <c r="F8" s="1">
-        <v>0.59632390024812099</v>
+        <v>0.65736861659606904</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
@@ -1744,16 +1744,16 @@
         <v>7</v>
       </c>
       <c r="C9" s="1">
-        <v>1.6039099443968701E-4</v>
+        <v>1.2208680538428301E-4</v>
       </c>
       <c r="D9" s="1">
-        <v>1.66294157162633E-4</v>
+        <v>1.6412918930395299E-4</v>
       </c>
       <c r="E9" s="1">
-        <v>0.96450168289934102</v>
+        <v>0.74384578332492202</v>
       </c>
       <c r="F9" s="1">
-        <v>0.34031531873463899</v>
+        <v>0.46111112883913302</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
@@ -1762,16 +1762,16 @@
         <v>10</v>
       </c>
       <c r="C10" s="1">
-        <v>-7.5215013217949395E-4</v>
+        <v>-5.75822963337933E-4</v>
       </c>
       <c r="D10" s="1">
-        <v>7.6897119614342802E-4</v>
+        <v>7.5896003307969495E-4</v>
       </c>
       <c r="E10" s="1">
-        <v>-0.97812523531662099</v>
+        <v>-0.75869998187041399</v>
       </c>
       <c r="F10" s="1">
-        <v>0.33361305843751698</v>
+        <v>0.45226893422200798</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
@@ -1782,16 +1782,16 @@
         <v>9</v>
       </c>
       <c r="C11" s="1">
-        <v>1.97028826221731E-4</v>
+        <v>2.5385914781209801E-4</v>
       </c>
       <c r="D11" s="1">
-        <v>5.8891870032100595E-4</v>
+        <v>5.9489217081268395E-4</v>
       </c>
       <c r="E11" s="1">
-        <v>0.33456031556534899</v>
+        <v>0.42673136455183103</v>
       </c>
       <c r="F11" s="1">
-        <v>0.73962183969531003</v>
+        <v>0.67175450921805402</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
@@ -1800,34 +1800,34 @@
         <v>8</v>
       </c>
       <c r="C12" s="1">
-        <v>-3.23386872814485E-3</v>
+        <v>-3.3335683574023801E-3</v>
       </c>
       <c r="D12" s="1">
-        <v>1.2484952226213099E-3</v>
+        <v>1.2611588540652899E-3</v>
       </c>
       <c r="E12" s="1">
-        <v>-2.5902131378245001</v>
+        <v>-2.6432581007989402</v>
       </c>
       <c r="F12" s="4">
-        <v>1.31293718725245E-2</v>
+        <v>1.14924654652948E-2</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" s="8"/>
-      <c r="B13" s="3" t="s">
+      <c r="B13" s="1" t="s">
         <v>7</v>
       </c>
       <c r="C13" s="1">
-        <v>3.2791453922484702E-4</v>
+        <v>2.9216342339675203E-4</v>
       </c>
       <c r="D13" s="1">
-        <v>1.91218155012373E-4</v>
+        <v>1.9315770287495001E-4</v>
       </c>
       <c r="E13" s="1">
-        <v>1.7148713687967001</v>
-      </c>
-      <c r="F13" s="3">
-        <v>9.3739580007072595E-2</v>
+        <v>1.51256418485106</v>
+      </c>
+      <c r="F13" s="1">
+        <v>0.137879322063552</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
@@ -1836,16 +1836,16 @@
         <v>10</v>
       </c>
       <c r="C14" s="1">
-        <v>-7.7661707932777098E-4</v>
+        <v>-6.00904070893631E-4</v>
       </c>
       <c r="D14" s="1">
-        <v>8.8422381094484205E-4</v>
+        <v>8.9319259532856E-4</v>
       </c>
       <c r="E14" s="1">
-        <v>-0.87830373907021597</v>
+        <v>-0.67275979899115601</v>
       </c>
       <c r="F14" s="1">
-        <v>0.38477599667599999</v>
+        <v>0.50478499720243697</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
@@ -1856,16 +1856,16 @@
         <v>9</v>
       </c>
       <c r="C15" s="2">
-        <v>-3.5825154663033903E-5</v>
+        <v>-3.7367131264075499E-5</v>
       </c>
       <c r="D15" s="2">
-        <v>1.8927460038076501E-5</v>
+        <v>1.9293464140715499E-5</v>
       </c>
       <c r="E15" s="1">
-        <v>-1.89276081370476</v>
+        <v>-1.93677667170297</v>
       </c>
       <c r="F15" s="3">
-        <v>6.5294653231981498E-2</v>
+        <v>5.9519120003501097E-2</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
@@ -1874,16 +1874,16 @@
         <v>8</v>
       </c>
       <c r="C16" s="2">
-        <v>-5.8390208894141502E-5</v>
+        <v>-5.8321131967602603E-5</v>
       </c>
       <c r="D16" s="2">
-        <v>4.0125816043901601E-5</v>
+        <v>4.0901737021373599E-5</v>
       </c>
       <c r="E16" s="1">
-        <v>-1.4551781035495199</v>
+        <v>-1.42588398964881</v>
       </c>
       <c r="F16" s="1">
-        <v>0.15305398014178601</v>
+        <v>0.161292513380344</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.25">
@@ -1892,16 +1892,16 @@
         <v>7</v>
       </c>
       <c r="C17" s="2">
-        <v>1.3575622868601501E-5</v>
+        <v>1.32400487650941E-5</v>
       </c>
       <c r="D17" s="2">
-        <v>6.1456258488287402E-6</v>
+        <v>6.2644650522628299E-6</v>
       </c>
       <c r="E17" s="1">
-        <v>2.2089894833394101</v>
+        <v>2.1135162627033202</v>
       </c>
       <c r="F17" s="4">
-        <v>3.2684032924149502E-2</v>
+        <v>4.0538433673404102E-2</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.25">
@@ -1910,16 +1910,16 @@
         <v>10</v>
       </c>
       <c r="C18" s="2">
-        <v>-3.0176903192067899E-5</v>
+        <v>-2.93095524997229E-5</v>
       </c>
       <c r="D18" s="2">
-        <v>2.84183722426402E-5</v>
+        <v>2.8967904023988802E-5</v>
       </c>
       <c r="E18" s="1">
-        <v>-1.06188007301801</v>
+        <v>-1.01179403506209</v>
       </c>
       <c r="F18" s="1">
-        <v>0.29435811396760603</v>
+        <v>0.317430198084722</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.25">
@@ -1930,16 +1930,16 @@
         <v>9</v>
       </c>
       <c r="C19" s="1">
-        <v>2.15160279809898E-3</v>
+        <v>2.10012764695973E-3</v>
       </c>
       <c r="D19" s="1">
-        <v>9.6063412902913897E-4</v>
+        <v>9.81861209707565E-4</v>
       </c>
       <c r="E19" s="1">
-        <v>2.2397734299462102</v>
+        <v>2.13892516192307</v>
       </c>
       <c r="F19" s="4">
-        <v>3.0456337762944499E-2</v>
+        <v>3.8300639855266501E-2</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.25">
@@ -1948,34 +1948,34 @@
         <v>8</v>
       </c>
       <c r="C20" s="1">
-        <v>-7.5561135023714298E-3</v>
+        <v>-7.3406351202516202E-3</v>
       </c>
       <c r="D20" s="1">
-        <v>2.03652409089086E-3</v>
+        <v>2.08152505418642E-3</v>
       </c>
       <c r="E20" s="1">
-        <v>-3.7102991003981001</v>
+        <v>-3.52656582513284</v>
       </c>
       <c r="F20" s="4">
-        <v>6.0210191906117001E-4</v>
+        <v>1.0330541069372701E-3</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A21" s="8"/>
-      <c r="B21" s="3" t="s">
+      <c r="B21" s="1" t="s">
         <v>7</v>
       </c>
       <c r="C21" s="1">
-        <v>-5.5751340316831095E-4</v>
+        <v>-4.5039893390444398E-4</v>
       </c>
       <c r="D21" s="1">
-        <v>3.1191178968292902E-4</v>
+        <v>3.18804087722395E-4</v>
       </c>
       <c r="E21" s="1">
-        <v>-1.7874072786252999</v>
-      </c>
-      <c r="F21" s="3">
-        <v>8.1089298193969594E-2</v>
+        <v>-1.41277653345724</v>
+      </c>
+      <c r="F21" s="1">
+        <v>0.16508940171310299</v>
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.25">
@@ -1983,17 +1983,17 @@
       <c r="B22" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="C22" s="2">
-        <v>3.5716593827619803E-5</v>
+      <c r="C22" s="1">
+        <v>-4.2286713246222099E-4</v>
       </c>
       <c r="D22" s="1">
-        <v>1.4423307835713601E-3</v>
+        <v>1.4742018893156401E-3</v>
       </c>
       <c r="E22" s="1">
-        <v>2.47631085978639E-2</v>
+        <v>-0.28684479074879399</v>
       </c>
       <c r="F22" s="1">
-        <v>0.98036120027870799</v>
+        <v>0.77564154544924002</v>
       </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.25">
@@ -2004,16 +2004,16 @@
         <v>9</v>
       </c>
       <c r="C23" s="1">
-        <v>5.8817294904817104E-3</v>
+        <v>5.5163316142661798E-3</v>
       </c>
       <c r="D23" s="1">
-        <v>6.2272802303673597E-3</v>
+        <v>6.38819386621818E-3</v>
       </c>
       <c r="E23" s="1">
-        <v>0.94451016702274404</v>
+        <v>0.86351975688112004</v>
       </c>
       <c r="F23" s="1">
-        <v>0.35031110487931999</v>
+        <v>0.392756411187282</v>
       </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.25">
@@ -2022,16 +2022,16 @@
         <v>8</v>
       </c>
       <c r="C24" s="1">
-        <v>-7.3045528780302498E-3</v>
+        <v>-7.4541826752963902E-3</v>
       </c>
       <c r="D24" s="1">
-        <v>1.3201702736387801E-2</v>
+        <v>1.3542836250241099E-2</v>
       </c>
       <c r="E24" s="1">
-        <v>-0.55330384450308201</v>
+        <v>-0.55041518169162695</v>
       </c>
       <c r="F24" s="1">
-        <v>0.58298890967638495</v>
+        <v>0.584950416090954</v>
       </c>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.25">
@@ -2040,16 +2040,16 @@
         <v>7</v>
       </c>
       <c r="C25" s="1">
-        <v>-9.2289269036274994E-3</v>
+        <v>-9.4486071792643997E-3</v>
       </c>
       <c r="D25" s="1">
-        <v>2.0219582698712199E-3</v>
+        <v>2.0742059036226298E-3</v>
       </c>
       <c r="E25" s="1">
-        <v>-4.5643508281777203</v>
+        <v>-4.5552889241913199</v>
       </c>
       <c r="F25" s="5">
-        <v>4.32123185112372E-5</v>
+        <v>4.44756348643138E-5</v>
       </c>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.25">
@@ -2058,16 +2058,16 @@
         <v>10</v>
       </c>
       <c r="C26" s="1">
-        <v>5.1637448869641103E-3</v>
+        <v>5.7352741689574898E-3</v>
       </c>
       <c r="D26" s="1">
-        <v>9.3498634940876301E-3</v>
+        <v>9.5914650398484392E-3</v>
       </c>
       <c r="E26" s="1">
-        <v>0.552280243474078</v>
+        <v>0.59795601038317703</v>
       </c>
       <c r="F26" s="1">
-        <v>0.58368360811750397</v>
+        <v>0.55308016139251204</v>
       </c>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.25">
@@ -2078,16 +2078,16 @@
         <v>9</v>
       </c>
       <c r="C27" s="1">
-        <v>1.8270517684183099E-2</v>
+        <v>1.8248054933923698E-2</v>
       </c>
       <c r="D27" s="1">
-        <v>4.4184348345621396E-3</v>
+        <v>4.5833998064322597E-3</v>
       </c>
       <c r="E27" s="1">
-        <v>4.1350655533643597</v>
+        <v>3.98133606156608</v>
       </c>
       <c r="F27" s="4">
-        <v>1.6614380889968299E-4</v>
+        <v>2.6631327356298797E-4</v>
       </c>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.25">
@@ -2096,16 +2096,16 @@
         <v>8</v>
       </c>
       <c r="C28" s="1">
-        <v>4.0722147842239403E-3</v>
+        <v>5.9298147427282203E-3</v>
       </c>
       <c r="D28" s="1">
-        <v>9.3669886512477308E-3</v>
+        <v>9.7167109120070497E-3</v>
       </c>
       <c r="E28" s="1">
-        <v>0.43474108230946801</v>
+        <v>0.610269750374139</v>
       </c>
       <c r="F28" s="1">
-        <v>0.66597601145868301</v>
+        <v>0.54497132192040398</v>
       </c>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.25">
@@ -2114,16 +2114,16 @@
         <v>7</v>
       </c>
       <c r="C29" s="1">
-        <v>-5.8861885046492099E-4</v>
+        <v>4.7143117990879502E-4</v>
       </c>
       <c r="D29" s="1">
-        <v>1.4346376785910201E-3</v>
+        <v>1.4882007553713599E-3</v>
       </c>
       <c r="E29" s="1">
-        <v>-0.41029094610355599</v>
+        <v>0.31677929083644002</v>
       </c>
       <c r="F29" s="1">
-        <v>0.68367806403607001</v>
+        <v>0.75298032999223496</v>
       </c>
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.25">
@@ -2132,16 +2132,16 @@
         <v>10</v>
       </c>
       <c r="C30" s="1">
-        <v>-4.5367957521503504E-3</v>
+        <v>-8.7325162942778391E-3</v>
       </c>
       <c r="D30" s="1">
-        <v>6.6339976735302003E-3</v>
+        <v>6.8816820415421101E-3</v>
       </c>
       <c r="E30" s="1">
-        <v>-0.68387056725272399</v>
+        <v>-1.2689508526495299</v>
       </c>
       <c r="F30" s="1">
-        <v>0.49781289740463303</v>
+        <v>0.21144617789143699</v>
       </c>
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.25">
@@ -2152,16 +2152,16 @@
         <v>9</v>
       </c>
       <c r="C31" s="1">
-        <v>1.5654496005932599E-2</v>
+        <v>1.5808279978672998E-2</v>
       </c>
       <c r="D31" s="1">
-        <v>4.2794975747358702E-3</v>
+        <v>4.3596069012505597E-3</v>
       </c>
       <c r="E31" s="1">
-        <v>3.6580219365818301</v>
+        <v>3.6260792169446199</v>
       </c>
       <c r="F31" s="4">
-        <v>7.0287164406071902E-4</v>
+        <v>7.7223464822892595E-4</v>
       </c>
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.25">
@@ -2170,16 +2170,16 @@
         <v>8</v>
       </c>
       <c r="C32" s="1">
-        <v>1.59394994363261E-2</v>
+        <v>1.5684132358793498E-2</v>
       </c>
       <c r="D32" s="1">
-        <v>9.0724445910189706E-3</v>
+        <v>9.24227467348448E-3</v>
       </c>
       <c r="E32" s="1">
-        <v>1.75691339598866</v>
+        <v>1.6969991601515899</v>
       </c>
       <c r="F32" s="3">
-        <v>8.6221150816636699E-2</v>
+        <v>9.7096827676740494E-2</v>
       </c>
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.25">
@@ -2188,16 +2188,16 @@
         <v>7</v>
       </c>
       <c r="C33" s="1">
-        <v>-5.8392474847676103E-4</v>
+        <v>-7.1537056274285199E-4</v>
       </c>
       <c r="D33" s="1">
-        <v>1.3895256343106001E-3</v>
+        <v>1.41553662293614E-3</v>
       </c>
       <c r="E33" s="1">
-        <v>-0.42023316019389001</v>
+        <v>-0.50537057900982596</v>
       </c>
       <c r="F33" s="1">
-        <v>0.67645737999211397</v>
+        <v>0.61594051398176997</v>
       </c>
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.25">
@@ -2206,29 +2206,29 @@
         <v>10</v>
       </c>
       <c r="C34" s="1">
-        <v>2.5105742368774402E-3</v>
+        <v>2.9704541726648299E-3</v>
       </c>
       <c r="D34" s="1">
-        <v>6.4253922526141096E-3</v>
+        <v>6.5456712893375698E-3</v>
       </c>
       <c r="E34" s="1">
-        <v>0.39072699971834901</v>
+        <v>0.45380436037224797</v>
       </c>
       <c r="F34" s="1">
-        <v>0.69797399323822196</v>
+        <v>0.65230597492016695</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="9">
+    <mergeCell ref="A31:A34"/>
+    <mergeCell ref="A27:A30"/>
+    <mergeCell ref="A23:A26"/>
+    <mergeCell ref="A11:A14"/>
     <mergeCell ref="A19:A22"/>
     <mergeCell ref="A15:A18"/>
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="A7:A10"/>
     <mergeCell ref="A3:A6"/>
-    <mergeCell ref="A31:A34"/>
-    <mergeCell ref="A27:A30"/>
-    <mergeCell ref="A23:A26"/>
-    <mergeCell ref="A11:A14"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>